<commit_message>
Updated calibration of allocation parameters and spatial prob perturbation process
</commit_message>
<xml_diff>
--- a/tools/lulc_class_aggregation.xlsx
+++ b/tools/lulc_class_aggregation.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="20394"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="20395"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\LULCC_CH\Tools\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C609C516-2716-4660-A79C-5057B69CF2F9}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E66D4054-41C7-4DE9-AE5B-60274C4B4B5F}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="21570" windowHeight="6480" xr2:uid="{461A3D3D-11BC-4F5B-AC99-BB9F607AA1FC}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="294" uniqueCount="231">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="367" uniqueCount="241">
   <si>
     <t>Industrie- und Gewerbegebäude</t>
   </si>
@@ -718,6 +718,36 @@
   </si>
   <si>
     <t>Glacier</t>
+  </si>
+  <si>
+    <t>Class_abbreviation</t>
+  </si>
+  <si>
+    <t>Urban</t>
+  </si>
+  <si>
+    <t>Static</t>
+  </si>
+  <si>
+    <t>Perm_crops</t>
+  </si>
+  <si>
+    <t>Int_AG</t>
+  </si>
+  <si>
+    <t>Grassland</t>
+  </si>
+  <si>
+    <t>Alp_Past</t>
+  </si>
+  <si>
+    <t>Closed_Forest</t>
+  </si>
+  <si>
+    <t>Open_Forest</t>
+  </si>
+  <si>
+    <t>Shrubland</t>
   </si>
 </sst>
 </file>
@@ -1181,14 +1211,14 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C6C81117-CCD0-4C70-9A30-E4F720811826}">
-  <dimension ref="A1:F73"/>
+  <dimension ref="A1:G73"/>
   <sheetFormatPr defaultColWidth="39.7109375" defaultRowHeight="12.75" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="14.28515625" style="5" customWidth="1"/>
     <col min="2" max="16384" width="39.7109375" style="5"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>144</v>
       </c>
@@ -1207,8 +1237,11 @@
       <c r="F1" s="8" t="s">
         <v>219</v>
       </c>
-    </row>
-    <row r="2" spans="1:6" ht="15" x14ac:dyDescent="0.25">
+      <c r="G1" s="5" t="s">
+        <v>231</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" ht="15" x14ac:dyDescent="0.25">
       <c r="A2" s="2">
         <v>1</v>
       </c>
@@ -1227,8 +1260,11 @@
       <c r="F2" s="9" t="s">
         <v>221</v>
       </c>
-    </row>
-    <row r="3" spans="1:6" ht="25.5" x14ac:dyDescent="0.25">
+      <c r="G2" s="5" t="s">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A3" s="2">
         <v>2</v>
       </c>
@@ -1247,8 +1283,11 @@
       <c r="F3" s="9" t="s">
         <v>221</v>
       </c>
-    </row>
-    <row r="4" spans="1:6" ht="25.5" x14ac:dyDescent="0.25">
+      <c r="G3" s="5" t="s">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A4" s="2">
         <v>3</v>
       </c>
@@ -1267,8 +1306,11 @@
       <c r="F4" s="9" t="s">
         <v>221</v>
       </c>
-    </row>
-    <row r="5" spans="1:6" ht="25.5" x14ac:dyDescent="0.25">
+      <c r="G4" s="5" t="s">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A5" s="2">
         <v>4</v>
       </c>
@@ -1287,8 +1329,11 @@
       <c r="F5" s="9" t="s">
         <v>221</v>
       </c>
-    </row>
-    <row r="6" spans="1:6" ht="15" x14ac:dyDescent="0.25">
+      <c r="G5" s="5" t="s">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" ht="15" x14ac:dyDescent="0.25">
       <c r="A6" s="2">
         <v>5</v>
       </c>
@@ -1307,8 +1352,11 @@
       <c r="F6" s="9" t="s">
         <v>221</v>
       </c>
-    </row>
-    <row r="7" spans="1:6" ht="25.5" x14ac:dyDescent="0.25">
+      <c r="G6" s="5" t="s">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A7" s="2">
         <v>6</v>
       </c>
@@ -1327,8 +1375,11 @@
       <c r="F7" s="9" t="s">
         <v>221</v>
       </c>
-    </row>
-    <row r="8" spans="1:6" ht="15" x14ac:dyDescent="0.25">
+      <c r="G7" s="5" t="s">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" ht="15" x14ac:dyDescent="0.25">
       <c r="A8" s="2">
         <v>7</v>
       </c>
@@ -1347,8 +1398,11 @@
       <c r="F8" s="9" t="s">
         <v>221</v>
       </c>
-    </row>
-    <row r="9" spans="1:6" ht="15" x14ac:dyDescent="0.25">
+      <c r="G8" s="5" t="s">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" ht="15" x14ac:dyDescent="0.25">
       <c r="A9" s="2">
         <v>8</v>
       </c>
@@ -1367,8 +1421,11 @@
       <c r="F9" s="9" t="s">
         <v>221</v>
       </c>
-    </row>
-    <row r="10" spans="1:6" ht="15" x14ac:dyDescent="0.25">
+      <c r="G9" s="5" t="s">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" ht="15" x14ac:dyDescent="0.25">
       <c r="A10" s="2">
         <v>9</v>
       </c>
@@ -1387,8 +1444,11 @@
       <c r="F10" s="9" t="s">
         <v>221</v>
       </c>
-    </row>
-    <row r="11" spans="1:6" ht="15" x14ac:dyDescent="0.25">
+      <c r="G10" s="5" t="s">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7" ht="15" x14ac:dyDescent="0.25">
       <c r="A11" s="2">
         <v>10</v>
       </c>
@@ -1407,8 +1467,11 @@
       <c r="F11" s="9" t="s">
         <v>221</v>
       </c>
-    </row>
-    <row r="12" spans="1:6" ht="15" x14ac:dyDescent="0.25">
+      <c r="G11" s="5" t="s">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7" ht="15" x14ac:dyDescent="0.25">
       <c r="A12" s="2">
         <v>11</v>
       </c>
@@ -1427,8 +1490,11 @@
       <c r="F12" s="9" t="s">
         <v>221</v>
       </c>
-    </row>
-    <row r="13" spans="1:6" ht="25.5" x14ac:dyDescent="0.25">
+      <c r="G12" s="5" t="s">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A13" s="2">
         <v>12</v>
       </c>
@@ -1447,8 +1513,11 @@
       <c r="F13" s="9" t="s">
         <v>221</v>
       </c>
-    </row>
-    <row r="14" spans="1:6" ht="15" x14ac:dyDescent="0.25">
+      <c r="G13" s="5" t="s">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="14" spans="1:7" ht="15" x14ac:dyDescent="0.25">
       <c r="A14" s="2">
         <v>13</v>
       </c>
@@ -1467,8 +1536,11 @@
       <c r="F14" s="9" t="s">
         <v>221</v>
       </c>
-    </row>
-    <row r="15" spans="1:6" ht="25.5" x14ac:dyDescent="0.25">
+      <c r="G14" s="5" t="s">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="15" spans="1:7" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A15" s="2">
         <v>14</v>
       </c>
@@ -1487,8 +1559,11 @@
       <c r="F15" s="9" t="s">
         <v>221</v>
       </c>
-    </row>
-    <row r="16" spans="1:6" ht="15" x14ac:dyDescent="0.25">
+      <c r="G15" s="5" t="s">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="16" spans="1:7" ht="15" x14ac:dyDescent="0.25">
       <c r="A16" s="2">
         <v>15</v>
       </c>
@@ -1507,8 +1582,11 @@
       <c r="F16" s="9" t="s">
         <v>222</v>
       </c>
-    </row>
-    <row r="17" spans="1:6" ht="15" x14ac:dyDescent="0.25">
+      <c r="G16" s="5" t="s">
+        <v>233</v>
+      </c>
+    </row>
+    <row r="17" spans="1:7" ht="15" x14ac:dyDescent="0.25">
       <c r="A17" s="2">
         <v>16</v>
       </c>
@@ -1527,8 +1605,11 @@
       <c r="F17" s="9" t="s">
         <v>222</v>
       </c>
-    </row>
-    <row r="18" spans="1:6" ht="15" x14ac:dyDescent="0.25">
+      <c r="G17" s="5" t="s">
+        <v>233</v>
+      </c>
+    </row>
+    <row r="18" spans="1:7" ht="15" x14ac:dyDescent="0.25">
       <c r="A18" s="2">
         <v>17</v>
       </c>
@@ -1547,8 +1628,11 @@
       <c r="F18" s="9" t="s">
         <v>222</v>
       </c>
-    </row>
-    <row r="19" spans="1:6" ht="15" x14ac:dyDescent="0.25">
+      <c r="G18" s="5" t="s">
+        <v>233</v>
+      </c>
+    </row>
+    <row r="19" spans="1:7" ht="15" x14ac:dyDescent="0.25">
       <c r="A19" s="2">
         <v>18</v>
       </c>
@@ -1567,8 +1651,11 @@
       <c r="F19" s="9" t="s">
         <v>222</v>
       </c>
-    </row>
-    <row r="20" spans="1:6" ht="15" x14ac:dyDescent="0.25">
+      <c r="G19" s="5" t="s">
+        <v>233</v>
+      </c>
+    </row>
+    <row r="20" spans="1:7" ht="15" x14ac:dyDescent="0.25">
       <c r="A20" s="2">
         <v>19</v>
       </c>
@@ -1587,8 +1674,11 @@
       <c r="F20" s="9" t="s">
         <v>221</v>
       </c>
-    </row>
-    <row r="21" spans="1:6" ht="15" x14ac:dyDescent="0.25">
+      <c r="G20" s="5" t="s">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="21" spans="1:7" ht="15" x14ac:dyDescent="0.25">
       <c r="A21" s="2">
         <v>20</v>
       </c>
@@ -1607,8 +1697,11 @@
       <c r="F21" s="9" t="s">
         <v>222</v>
       </c>
-    </row>
-    <row r="22" spans="1:6" ht="15" x14ac:dyDescent="0.25">
+      <c r="G21" s="5" t="s">
+        <v>233</v>
+      </c>
+    </row>
+    <row r="22" spans="1:7" ht="15" x14ac:dyDescent="0.25">
       <c r="A22" s="2">
         <v>21</v>
       </c>
@@ -1627,8 +1720,11 @@
       <c r="F22" s="9" t="s">
         <v>222</v>
       </c>
-    </row>
-    <row r="23" spans="1:6" ht="15" x14ac:dyDescent="0.25">
+      <c r="G22" s="5" t="s">
+        <v>233</v>
+      </c>
+    </row>
+    <row r="23" spans="1:7" ht="15" x14ac:dyDescent="0.25">
       <c r="A23" s="2">
         <v>22</v>
       </c>
@@ -1647,8 +1743,11 @@
       <c r="F23" s="9" t="s">
         <v>222</v>
       </c>
-    </row>
-    <row r="24" spans="1:6" ht="15" x14ac:dyDescent="0.25">
+      <c r="G23" s="5" t="s">
+        <v>233</v>
+      </c>
+    </row>
+    <row r="24" spans="1:7" ht="15" x14ac:dyDescent="0.25">
       <c r="A24" s="2">
         <v>23</v>
       </c>
@@ -1667,8 +1766,11 @@
       <c r="F24" s="9" t="s">
         <v>222</v>
       </c>
-    </row>
-    <row r="25" spans="1:6" ht="15" x14ac:dyDescent="0.25">
+      <c r="G24" s="5" t="s">
+        <v>233</v>
+      </c>
+    </row>
+    <row r="25" spans="1:7" ht="15" x14ac:dyDescent="0.25">
       <c r="A25" s="2">
         <v>24</v>
       </c>
@@ -1687,8 +1789,11 @@
       <c r="F25" s="9" t="s">
         <v>222</v>
       </c>
-    </row>
-    <row r="26" spans="1:6" ht="15" x14ac:dyDescent="0.25">
+      <c r="G25" s="5" t="s">
+        <v>233</v>
+      </c>
+    </row>
+    <row r="26" spans="1:7" ht="15" x14ac:dyDescent="0.25">
       <c r="A26" s="2">
         <v>25</v>
       </c>
@@ -1707,8 +1812,11 @@
       <c r="F26" s="9" t="s">
         <v>222</v>
       </c>
-    </row>
-    <row r="27" spans="1:6" ht="25.5" x14ac:dyDescent="0.25">
+      <c r="G26" s="5" t="s">
+        <v>233</v>
+      </c>
+    </row>
+    <row r="27" spans="1:7" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A27" s="2">
         <v>26</v>
       </c>
@@ -1727,8 +1835,11 @@
       <c r="F27" s="9" t="s">
         <v>222</v>
       </c>
-    </row>
-    <row r="28" spans="1:6" ht="15" x14ac:dyDescent="0.25">
+      <c r="G27" s="5" t="s">
+        <v>233</v>
+      </c>
+    </row>
+    <row r="28" spans="1:7" ht="15" x14ac:dyDescent="0.25">
       <c r="A28" s="2">
         <v>27</v>
       </c>
@@ -1747,8 +1858,11 @@
       <c r="F28" s="9" t="s">
         <v>222</v>
       </c>
-    </row>
-    <row r="29" spans="1:6" ht="15" x14ac:dyDescent="0.25">
+      <c r="G28" s="5" t="s">
+        <v>233</v>
+      </c>
+    </row>
+    <row r="29" spans="1:7" ht="15" x14ac:dyDescent="0.25">
       <c r="A29" s="2">
         <v>28</v>
       </c>
@@ -1767,8 +1881,11 @@
       <c r="F29" s="9" t="s">
         <v>222</v>
       </c>
-    </row>
-    <row r="30" spans="1:6" ht="15" x14ac:dyDescent="0.25">
+      <c r="G29" s="5" t="s">
+        <v>233</v>
+      </c>
+    </row>
+    <row r="30" spans="1:7" ht="15" x14ac:dyDescent="0.25">
       <c r="A30" s="2">
         <v>29</v>
       </c>
@@ -1787,8 +1904,11 @@
       <c r="F30" s="9" t="s">
         <v>221</v>
       </c>
-    </row>
-    <row r="31" spans="1:6" ht="15" x14ac:dyDescent="0.25">
+      <c r="G30" s="5" t="s">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="31" spans="1:7" ht="15" x14ac:dyDescent="0.25">
       <c r="A31" s="2">
         <v>30</v>
       </c>
@@ -1807,8 +1927,11 @@
       <c r="F31" s="9" t="s">
         <v>221</v>
       </c>
-    </row>
-    <row r="32" spans="1:6" ht="15" x14ac:dyDescent="0.25">
+      <c r="G31" s="5" t="s">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="32" spans="1:7" ht="15" x14ac:dyDescent="0.25">
       <c r="A32" s="2">
         <v>31</v>
       </c>
@@ -1827,8 +1950,11 @@
       <c r="F32" s="9" t="s">
         <v>221</v>
       </c>
-    </row>
-    <row r="33" spans="1:6" ht="15" x14ac:dyDescent="0.25">
+      <c r="G32" s="5" t="s">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="33" spans="1:7" ht="15" x14ac:dyDescent="0.25">
       <c r="A33" s="2">
         <v>32</v>
       </c>
@@ -1847,8 +1973,11 @@
       <c r="F33" s="9" t="s">
         <v>221</v>
       </c>
-    </row>
-    <row r="34" spans="1:6" ht="15" x14ac:dyDescent="0.25">
+      <c r="G33" s="5" t="s">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="34" spans="1:7" ht="15" x14ac:dyDescent="0.25">
       <c r="A34" s="2">
         <v>33</v>
       </c>
@@ -1867,8 +1996,11 @@
       <c r="F34" s="9" t="s">
         <v>221</v>
       </c>
-    </row>
-    <row r="35" spans="1:6" ht="15" x14ac:dyDescent="0.25">
+      <c r="G34" s="5" t="s">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="35" spans="1:7" ht="15" x14ac:dyDescent="0.25">
       <c r="A35" s="2">
         <v>34</v>
       </c>
@@ -1887,8 +2019,11 @@
       <c r="F35" s="9" t="s">
         <v>221</v>
       </c>
-    </row>
-    <row r="36" spans="1:6" ht="15" x14ac:dyDescent="0.25">
+      <c r="G35" s="5" t="s">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="36" spans="1:7" ht="15" x14ac:dyDescent="0.25">
       <c r="A36" s="2">
         <v>35</v>
       </c>
@@ -1907,8 +2042,11 @@
       <c r="F36" s="9" t="s">
         <v>221</v>
       </c>
-    </row>
-    <row r="37" spans="1:6" ht="15" x14ac:dyDescent="0.25">
+      <c r="G36" s="5" t="s">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="37" spans="1:7" ht="15" x14ac:dyDescent="0.25">
       <c r="A37" s="2">
         <v>36</v>
       </c>
@@ -1927,8 +2065,11 @@
       <c r="F37" s="9" t="s">
         <v>221</v>
       </c>
-    </row>
-    <row r="38" spans="1:6" ht="15" x14ac:dyDescent="0.25">
+      <c r="G37" s="5" t="s">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="38" spans="1:7" ht="15" x14ac:dyDescent="0.25">
       <c r="A38" s="2">
         <v>37</v>
       </c>
@@ -1947,8 +2088,11 @@
       <c r="F38" s="9" t="s">
         <v>223</v>
       </c>
-    </row>
-    <row r="39" spans="1:6" ht="15" x14ac:dyDescent="0.25">
+      <c r="G38" s="5" t="s">
+        <v>234</v>
+      </c>
+    </row>
+    <row r="39" spans="1:7" ht="15" x14ac:dyDescent="0.25">
       <c r="A39" s="2">
         <v>38</v>
       </c>
@@ -1967,8 +2111,11 @@
       <c r="F39" s="9" t="s">
         <v>223</v>
       </c>
-    </row>
-    <row r="40" spans="1:6" ht="15" x14ac:dyDescent="0.25">
+      <c r="G39" s="5" t="s">
+        <v>234</v>
+      </c>
+    </row>
+    <row r="40" spans="1:7" ht="15" x14ac:dyDescent="0.25">
       <c r="A40" s="2">
         <v>39</v>
       </c>
@@ -1987,8 +2134,11 @@
       <c r="F40" s="9" t="s">
         <v>223</v>
       </c>
-    </row>
-    <row r="41" spans="1:6" ht="15" x14ac:dyDescent="0.25">
+      <c r="G40" s="5" t="s">
+        <v>234</v>
+      </c>
+    </row>
+    <row r="41" spans="1:7" ht="15" x14ac:dyDescent="0.25">
       <c r="A41" s="2">
         <v>40</v>
       </c>
@@ -2007,8 +2157,11 @@
       <c r="F41" s="9" t="s">
         <v>223</v>
       </c>
-    </row>
-    <row r="42" spans="1:6" ht="15" x14ac:dyDescent="0.25">
+      <c r="G41" s="5" t="s">
+        <v>234</v>
+      </c>
+    </row>
+    <row r="42" spans="1:7" ht="15" x14ac:dyDescent="0.25">
       <c r="A42" s="2">
         <v>41</v>
       </c>
@@ -2027,8 +2180,11 @@
       <c r="F42" s="9" t="s">
         <v>224</v>
       </c>
-    </row>
-    <row r="43" spans="1:6" ht="15" x14ac:dyDescent="0.25">
+      <c r="G42" s="5" t="s">
+        <v>235</v>
+      </c>
+    </row>
+    <row r="43" spans="1:7" ht="15" x14ac:dyDescent="0.25">
       <c r="A43" s="2">
         <v>42</v>
       </c>
@@ -2047,8 +2203,11 @@
       <c r="F43" s="9" t="s">
         <v>225</v>
       </c>
-    </row>
-    <row r="44" spans="1:6" ht="15" x14ac:dyDescent="0.25">
+      <c r="G43" s="5" t="s">
+        <v>236</v>
+      </c>
+    </row>
+    <row r="44" spans="1:7" ht="15" x14ac:dyDescent="0.25">
       <c r="A44" s="2">
         <v>43</v>
       </c>
@@ -2067,8 +2226,11 @@
       <c r="F44" s="9" t="s">
         <v>225</v>
       </c>
-    </row>
-    <row r="45" spans="1:6" ht="15" x14ac:dyDescent="0.25">
+      <c r="G44" s="5" t="s">
+        <v>236</v>
+      </c>
+    </row>
+    <row r="45" spans="1:7" ht="15" x14ac:dyDescent="0.25">
       <c r="A45" s="2">
         <v>44</v>
       </c>
@@ -2087,8 +2249,11 @@
       <c r="F45" s="9" t="s">
         <v>225</v>
       </c>
-    </row>
-    <row r="46" spans="1:6" ht="15" x14ac:dyDescent="0.25">
+      <c r="G45" s="5" t="s">
+        <v>236</v>
+      </c>
+    </row>
+    <row r="46" spans="1:7" ht="15" x14ac:dyDescent="0.25">
       <c r="A46" s="2">
         <v>45</v>
       </c>
@@ -2107,8 +2272,11 @@
       <c r="F46" s="9" t="s">
         <v>225</v>
       </c>
-    </row>
-    <row r="47" spans="1:6" ht="15" x14ac:dyDescent="0.25">
+      <c r="G46" s="5" t="s">
+        <v>236</v>
+      </c>
+    </row>
+    <row r="47" spans="1:7" ht="15" x14ac:dyDescent="0.25">
       <c r="A47" s="2">
         <v>46</v>
       </c>
@@ -2127,8 +2295,11 @@
       <c r="F47" s="9" t="s">
         <v>226</v>
       </c>
-    </row>
-    <row r="48" spans="1:6" ht="15" x14ac:dyDescent="0.25">
+      <c r="G47" s="5" t="s">
+        <v>237</v>
+      </c>
+    </row>
+    <row r="48" spans="1:7" ht="15" x14ac:dyDescent="0.25">
       <c r="A48" s="2">
         <v>47</v>
       </c>
@@ -2147,8 +2318,11 @@
       <c r="F48" s="9" t="s">
         <v>226</v>
       </c>
-    </row>
-    <row r="49" spans="1:6" ht="15" x14ac:dyDescent="0.25">
+      <c r="G48" s="5" t="s">
+        <v>237</v>
+      </c>
+    </row>
+    <row r="49" spans="1:7" ht="15" x14ac:dyDescent="0.25">
       <c r="A49" s="2">
         <v>48</v>
       </c>
@@ -2167,8 +2341,11 @@
       <c r="F49" s="9" t="s">
         <v>226</v>
       </c>
-    </row>
-    <row r="50" spans="1:6" ht="15" x14ac:dyDescent="0.25">
+      <c r="G49" s="5" t="s">
+        <v>237</v>
+      </c>
+    </row>
+    <row r="50" spans="1:7" ht="15" x14ac:dyDescent="0.25">
       <c r="A50" s="2">
         <v>49</v>
       </c>
@@ -2187,8 +2364,11 @@
       <c r="F50" s="9" t="s">
         <v>226</v>
       </c>
-    </row>
-    <row r="51" spans="1:6" ht="15" x14ac:dyDescent="0.25">
+      <c r="G50" s="5" t="s">
+        <v>237</v>
+      </c>
+    </row>
+    <row r="51" spans="1:7" ht="15" x14ac:dyDescent="0.25">
       <c r="A51" s="2">
         <v>50</v>
       </c>
@@ -2207,8 +2387,11 @@
       <c r="F51" s="9" t="s">
         <v>227</v>
       </c>
-    </row>
-    <row r="52" spans="1:6" ht="15" x14ac:dyDescent="0.25">
+      <c r="G51" s="5" t="s">
+        <v>238</v>
+      </c>
+    </row>
+    <row r="52" spans="1:7" ht="15" x14ac:dyDescent="0.25">
       <c r="A52" s="2">
         <v>51</v>
       </c>
@@ -2227,8 +2410,11 @@
       <c r="F52" s="9" t="s">
         <v>227</v>
       </c>
-    </row>
-    <row r="53" spans="1:6" ht="15" x14ac:dyDescent="0.25">
+      <c r="G52" s="5" t="s">
+        <v>238</v>
+      </c>
+    </row>
+    <row r="53" spans="1:7" ht="15" x14ac:dyDescent="0.25">
       <c r="A53" s="2">
         <v>52</v>
       </c>
@@ -2247,8 +2433,11 @@
       <c r="F53" s="9" t="s">
         <v>227</v>
       </c>
-    </row>
-    <row r="54" spans="1:6" ht="15" x14ac:dyDescent="0.25">
+      <c r="G53" s="5" t="s">
+        <v>238</v>
+      </c>
+    </row>
+    <row r="54" spans="1:7" ht="15" x14ac:dyDescent="0.25">
       <c r="A54" s="2">
         <v>53</v>
       </c>
@@ -2267,8 +2456,11 @@
       <c r="F54" s="9" t="s">
         <v>227</v>
       </c>
-    </row>
-    <row r="55" spans="1:6" ht="15" x14ac:dyDescent="0.25">
+      <c r="G54" s="5" t="s">
+        <v>238</v>
+      </c>
+    </row>
+    <row r="55" spans="1:7" ht="15" x14ac:dyDescent="0.25">
       <c r="A55" s="2">
         <v>54</v>
       </c>
@@ -2287,8 +2479,11 @@
       <c r="F55" s="9" t="s">
         <v>228</v>
       </c>
-    </row>
-    <row r="56" spans="1:6" ht="15" x14ac:dyDescent="0.25">
+      <c r="G55" s="5" t="s">
+        <v>239</v>
+      </c>
+    </row>
+    <row r="56" spans="1:7" ht="15" x14ac:dyDescent="0.25">
       <c r="A56" s="2">
         <v>55</v>
       </c>
@@ -2307,8 +2502,11 @@
       <c r="F56" s="9" t="s">
         <v>228</v>
       </c>
-    </row>
-    <row r="57" spans="1:6" ht="15" x14ac:dyDescent="0.25">
+      <c r="G56" s="5" t="s">
+        <v>239</v>
+      </c>
+    </row>
+    <row r="57" spans="1:7" ht="15" x14ac:dyDescent="0.25">
       <c r="A57" s="2">
         <v>56</v>
       </c>
@@ -2327,8 +2525,11 @@
       <c r="F57" s="9" t="s">
         <v>228</v>
       </c>
-    </row>
-    <row r="58" spans="1:6" ht="15" x14ac:dyDescent="0.25">
+      <c r="G57" s="5" t="s">
+        <v>239</v>
+      </c>
+    </row>
+    <row r="58" spans="1:7" ht="15" x14ac:dyDescent="0.25">
       <c r="A58" s="2">
         <v>57</v>
       </c>
@@ -2347,8 +2548,11 @@
       <c r="F58" s="9" t="s">
         <v>227</v>
       </c>
-    </row>
-    <row r="59" spans="1:6" ht="15" x14ac:dyDescent="0.25">
+      <c r="G58" s="5" t="s">
+        <v>238</v>
+      </c>
+    </row>
+    <row r="59" spans="1:7" ht="15" x14ac:dyDescent="0.25">
       <c r="A59" s="2">
         <v>58</v>
       </c>
@@ -2367,8 +2571,11 @@
       <c r="F59" s="9" t="s">
         <v>228</v>
       </c>
-    </row>
-    <row r="60" spans="1:6" ht="15" x14ac:dyDescent="0.25">
+      <c r="G59" s="5" t="s">
+        <v>239</v>
+      </c>
+    </row>
+    <row r="60" spans="1:7" ht="15" x14ac:dyDescent="0.25">
       <c r="A60" s="2">
         <v>59</v>
       </c>
@@ -2387,8 +2594,11 @@
       <c r="F60" s="9" t="s">
         <v>228</v>
       </c>
-    </row>
-    <row r="61" spans="1:6" ht="15" x14ac:dyDescent="0.25">
+      <c r="G60" s="5" t="s">
+        <v>239</v>
+      </c>
+    </row>
+    <row r="61" spans="1:7" ht="15" x14ac:dyDescent="0.25">
       <c r="A61" s="2">
         <v>60</v>
       </c>
@@ -2407,8 +2617,11 @@
       <c r="F61" s="9" t="s">
         <v>228</v>
       </c>
-    </row>
-    <row r="62" spans="1:6" ht="15" x14ac:dyDescent="0.25">
+      <c r="G61" s="5" t="s">
+        <v>239</v>
+      </c>
+    </row>
+    <row r="62" spans="1:7" ht="15" x14ac:dyDescent="0.25">
       <c r="A62" s="2">
         <v>61</v>
       </c>
@@ -2427,8 +2640,11 @@
       <c r="F62" s="9" t="s">
         <v>222</v>
       </c>
-    </row>
-    <row r="63" spans="1:6" ht="15" x14ac:dyDescent="0.25">
+      <c r="G62" s="5" t="s">
+        <v>233</v>
+      </c>
+    </row>
+    <row r="63" spans="1:7" ht="15" x14ac:dyDescent="0.25">
       <c r="A63" s="2">
         <v>62</v>
       </c>
@@ -2447,8 +2663,11 @@
       <c r="F63" s="9" t="s">
         <v>222</v>
       </c>
-    </row>
-    <row r="64" spans="1:6" ht="15" x14ac:dyDescent="0.25">
+      <c r="G63" s="5" t="s">
+        <v>233</v>
+      </c>
+    </row>
+    <row r="64" spans="1:7" ht="15" x14ac:dyDescent="0.25">
       <c r="A64" s="2">
         <v>63</v>
       </c>
@@ -2467,8 +2686,11 @@
       <c r="F64" s="9" t="s">
         <v>222</v>
       </c>
-    </row>
-    <row r="65" spans="1:6" ht="15" x14ac:dyDescent="0.25">
+      <c r="G64" s="5" t="s">
+        <v>233</v>
+      </c>
+    </row>
+    <row r="65" spans="1:7" ht="15" x14ac:dyDescent="0.25">
       <c r="A65" s="2">
         <v>64</v>
       </c>
@@ -2487,8 +2709,11 @@
       <c r="F65" s="9" t="s">
         <v>229</v>
       </c>
-    </row>
-    <row r="66" spans="1:6" ht="15" x14ac:dyDescent="0.25">
+      <c r="G65" s="5" t="s">
+        <v>240</v>
+      </c>
+    </row>
+    <row r="66" spans="1:7" ht="15" x14ac:dyDescent="0.25">
       <c r="A66" s="2">
         <v>65</v>
       </c>
@@ -2507,8 +2732,11 @@
       <c r="F66" s="9" t="s">
         <v>229</v>
       </c>
-    </row>
-    <row r="67" spans="1:6" ht="25.5" x14ac:dyDescent="0.25">
+      <c r="G66" s="5" t="s">
+        <v>240</v>
+      </c>
+    </row>
+    <row r="67" spans="1:7" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A67" s="2">
         <v>66</v>
       </c>
@@ -2527,8 +2755,11 @@
       <c r="F67" s="9" t="s">
         <v>222</v>
       </c>
-    </row>
-    <row r="68" spans="1:6" ht="15" x14ac:dyDescent="0.25">
+      <c r="G67" s="5" t="s">
+        <v>233</v>
+      </c>
+    </row>
+    <row r="68" spans="1:7" ht="15" x14ac:dyDescent="0.25">
       <c r="A68" s="2">
         <v>67</v>
       </c>
@@ -2547,8 +2778,11 @@
       <c r="F68" s="9" t="s">
         <v>222</v>
       </c>
-    </row>
-    <row r="69" spans="1:6" ht="15" x14ac:dyDescent="0.25">
+      <c r="G68" s="5" t="s">
+        <v>233</v>
+      </c>
+    </row>
+    <row r="69" spans="1:7" ht="15" x14ac:dyDescent="0.25">
       <c r="A69" s="2">
         <v>68</v>
       </c>
@@ -2567,8 +2801,11 @@
       <c r="F69" s="9" t="s">
         <v>222</v>
       </c>
-    </row>
-    <row r="70" spans="1:6" ht="15" x14ac:dyDescent="0.25">
+      <c r="G69" s="5" t="s">
+        <v>233</v>
+      </c>
+    </row>
+    <row r="70" spans="1:7" ht="15" x14ac:dyDescent="0.25">
       <c r="A70" s="2">
         <v>69</v>
       </c>
@@ -2587,8 +2824,11 @@
       <c r="F70" s="9" t="s">
         <v>222</v>
       </c>
-    </row>
-    <row r="71" spans="1:6" ht="15" x14ac:dyDescent="0.25">
+      <c r="G70" s="5" t="s">
+        <v>233</v>
+      </c>
+    </row>
+    <row r="71" spans="1:7" ht="15" x14ac:dyDescent="0.25">
       <c r="A71" s="2">
         <v>70</v>
       </c>
@@ -2607,8 +2847,11 @@
       <c r="F71" s="9" t="s">
         <v>222</v>
       </c>
-    </row>
-    <row r="72" spans="1:6" ht="15" x14ac:dyDescent="0.25">
+      <c r="G71" s="5" t="s">
+        <v>233</v>
+      </c>
+    </row>
+    <row r="72" spans="1:7" ht="15" x14ac:dyDescent="0.25">
       <c r="A72" s="2">
         <v>71</v>
       </c>
@@ -2627,8 +2870,11 @@
       <c r="F72" s="9" t="s">
         <v>222</v>
       </c>
-    </row>
-    <row r="73" spans="1:6" ht="15" x14ac:dyDescent="0.25">
+      <c r="G72" s="5" t="s">
+        <v>233</v>
+      </c>
+    </row>
+    <row r="73" spans="1:7" ht="15" x14ac:dyDescent="0.25">
       <c r="A73" s="2">
         <v>72</v>
       </c>
@@ -2645,6 +2891,9 @@
         <v>19</v>
       </c>
       <c r="F73" s="9" t="s">
+        <v>230</v>
+      </c>
+      <c r="G73" s="5" t="s">
         <v>230</v>
       </c>
     </row>

</xml_diff>

<commit_message>
All scripts following first complete run of simulations
</commit_message>
<xml_diff>
--- a/tools/lulc_class_aggregation.xlsx
+++ b/tools/lulc_class_aggregation.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="20395"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="20398"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\LULCC_CH\Tools\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E66D4054-41C7-4DE9-AE5B-60274C4B4B5F}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{16AFE05E-97B3-4278-AD2A-D844CE6A9FEA}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="21570" windowHeight="6480" xr2:uid="{461A3D3D-11BC-4F5B-AC99-BB9F607AA1FC}"/>
   </bookViews>

</xml_diff>

<commit_message>
Long test, Reduce log output, ignore model backups
squash! Long test, Reduce log output, ignore model backups
</commit_message>
<xml_diff>
--- a/tools/lulc_class_aggregation.xlsx
+++ b/tools/lulc_class_aggregation.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="20398"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="26924"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\LULCC_CH\Tools\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\bblack\switchdrive\C.3_Modelling\LULCC_CH_HPC\Tools\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{16AFE05E-97B3-4278-AD2A-D844CE6A9FEA}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FB7150C2-BB2F-41DF-8002-A52E3EBAB9A4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="21570" windowHeight="6480" xr2:uid="{461A3D3D-11BC-4F5B-AC99-BB9F607AA1FC}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{461A3D3D-11BC-4F5B-AC99-BB9F607AA1FC}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -877,7 +877,7 @@
     <xf numFmtId="0" fontId="5" fillId="2" borderId="1" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">

</xml_diff>

<commit_message>
- Update Dinamica model to source scripts - Update to scenario specifications management
</commit_message>
<xml_diff>
--- a/tools/lulc_class_aggregation.xlsx
+++ b/tools/lulc_class_aggregation.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="26731"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="26924"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\bblack\switchdrive\C.3_Modelling\LULCC_CH\Tools\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\bblack\switchdrive\C.3_Modelling\LULCC_CH_HPC\Tools\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0CEC9D1C-D943-4799-89AF-FEF1303BBCEB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FB7150C2-BB2F-41DF-8002-A52E3EBAB9A4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-98" yWindow="-98" windowWidth="19396" windowHeight="10395" xr2:uid="{461A3D3D-11BC-4F5B-AC99-BB9F607AA1FC}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{461A3D3D-11BC-4F5B-AC99-BB9F607AA1FC}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="440" uniqueCount="244">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="367" uniqueCount="241">
   <si>
     <t>Industrie- und Gewerbegebäude</t>
   </si>
@@ -748,15 +748,6 @@
   </si>
   <si>
     <t>Shrubland</t>
-  </si>
-  <si>
-    <t>Aggregated_class_short</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Urban/amenities </t>
-  </si>
-  <si>
-    <t>Overgrown/shrubland</t>
   </si>
 </sst>
 </file>
@@ -1220,14 +1211,14 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C6C81117-CCD0-4C70-9A30-E4F720811826}">
-  <dimension ref="A1:H73"/>
-  <sheetFormatPr defaultColWidth="39.73046875" defaultRowHeight="13.15" x14ac:dyDescent="0.45"/>
+  <dimension ref="A1:G73"/>
+  <sheetFormatPr defaultColWidth="39.7109375" defaultRowHeight="12.75" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="14.265625" style="5" customWidth="1"/>
-    <col min="2" max="16384" width="39.73046875" style="5"/>
+    <col min="1" max="1" width="14.28515625" style="5" customWidth="1"/>
+    <col min="2" max="16384" width="39.7109375" style="5"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.45">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>144</v>
       </c>
@@ -1246,14 +1237,11 @@
       <c r="F1" s="8" t="s">
         <v>219</v>
       </c>
-      <c r="G1" s="8" t="s">
-        <v>241</v>
-      </c>
-      <c r="H1" s="5" t="s">
+      <c r="G1" s="5" t="s">
         <v>231</v>
       </c>
     </row>
-    <row r="2" spans="1:8" ht="14.25" x14ac:dyDescent="0.45">
+    <row r="2" spans="1:7" ht="15" x14ac:dyDescent="0.25">
       <c r="A2" s="2">
         <v>1</v>
       </c>
@@ -1272,14 +1260,11 @@
       <c r="F2" s="9" t="s">
         <v>221</v>
       </c>
-      <c r="G2" s="9" t="s">
-        <v>242</v>
-      </c>
-      <c r="H2" s="5" t="s">
+      <c r="G2" s="5" t="s">
         <v>232</v>
       </c>
     </row>
-    <row r="3" spans="1:8" ht="26.25" x14ac:dyDescent="0.45">
+    <row r="3" spans="1:7" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A3" s="2">
         <v>2</v>
       </c>
@@ -1298,14 +1283,11 @@
       <c r="F3" s="9" t="s">
         <v>221</v>
       </c>
-      <c r="G3" s="9" t="s">
-        <v>242</v>
-      </c>
-      <c r="H3" s="5" t="s">
+      <c r="G3" s="5" t="s">
         <v>232</v>
       </c>
     </row>
-    <row r="4" spans="1:8" ht="14.25" x14ac:dyDescent="0.45">
+    <row r="4" spans="1:7" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A4" s="2">
         <v>3</v>
       </c>
@@ -1324,14 +1306,11 @@
       <c r="F4" s="9" t="s">
         <v>221</v>
       </c>
-      <c r="G4" s="9" t="s">
-        <v>242</v>
-      </c>
-      <c r="H4" s="5" t="s">
+      <c r="G4" s="5" t="s">
         <v>232</v>
       </c>
     </row>
-    <row r="5" spans="1:8" ht="26.25" x14ac:dyDescent="0.45">
+    <row r="5" spans="1:7" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A5" s="2">
         <v>4</v>
       </c>
@@ -1350,14 +1329,11 @@
       <c r="F5" s="9" t="s">
         <v>221</v>
       </c>
-      <c r="G5" s="9" t="s">
-        <v>242</v>
-      </c>
-      <c r="H5" s="5" t="s">
+      <c r="G5" s="5" t="s">
         <v>232</v>
       </c>
     </row>
-    <row r="6" spans="1:8" ht="14.25" x14ac:dyDescent="0.45">
+    <row r="6" spans="1:7" ht="15" x14ac:dyDescent="0.25">
       <c r="A6" s="2">
         <v>5</v>
       </c>
@@ -1376,14 +1352,11 @@
       <c r="F6" s="9" t="s">
         <v>221</v>
       </c>
-      <c r="G6" s="9" t="s">
-        <v>242</v>
-      </c>
-      <c r="H6" s="5" t="s">
+      <c r="G6" s="5" t="s">
         <v>232</v>
       </c>
     </row>
-    <row r="7" spans="1:8" ht="26.25" x14ac:dyDescent="0.45">
+    <row r="7" spans="1:7" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A7" s="2">
         <v>6</v>
       </c>
@@ -1402,14 +1375,11 @@
       <c r="F7" s="9" t="s">
         <v>221</v>
       </c>
-      <c r="G7" s="9" t="s">
-        <v>242</v>
-      </c>
-      <c r="H7" s="5" t="s">
+      <c r="G7" s="5" t="s">
         <v>232</v>
       </c>
     </row>
-    <row r="8" spans="1:8" ht="14.25" x14ac:dyDescent="0.45">
+    <row r="8" spans="1:7" ht="15" x14ac:dyDescent="0.25">
       <c r="A8" s="2">
         <v>7</v>
       </c>
@@ -1428,14 +1398,11 @@
       <c r="F8" s="9" t="s">
         <v>221</v>
       </c>
-      <c r="G8" s="9" t="s">
-        <v>242</v>
-      </c>
-      <c r="H8" s="5" t="s">
+      <c r="G8" s="5" t="s">
         <v>232</v>
       </c>
     </row>
-    <row r="9" spans="1:8" ht="14.25" x14ac:dyDescent="0.45">
+    <row r="9" spans="1:7" ht="15" x14ac:dyDescent="0.25">
       <c r="A9" s="2">
         <v>8</v>
       </c>
@@ -1454,14 +1421,11 @@
       <c r="F9" s="9" t="s">
         <v>221</v>
       </c>
-      <c r="G9" s="9" t="s">
-        <v>242</v>
-      </c>
-      <c r="H9" s="5" t="s">
+      <c r="G9" s="5" t="s">
         <v>232</v>
       </c>
     </row>
-    <row r="10" spans="1:8" ht="14.25" x14ac:dyDescent="0.45">
+    <row r="10" spans="1:7" ht="15" x14ac:dyDescent="0.25">
       <c r="A10" s="2">
         <v>9</v>
       </c>
@@ -1480,14 +1444,11 @@
       <c r="F10" s="9" t="s">
         <v>221</v>
       </c>
-      <c r="G10" s="9" t="s">
-        <v>242</v>
-      </c>
-      <c r="H10" s="5" t="s">
+      <c r="G10" s="5" t="s">
         <v>232</v>
       </c>
     </row>
-    <row r="11" spans="1:8" ht="14.25" x14ac:dyDescent="0.45">
+    <row r="11" spans="1:7" ht="15" x14ac:dyDescent="0.25">
       <c r="A11" s="2">
         <v>10</v>
       </c>
@@ -1506,14 +1467,11 @@
       <c r="F11" s="9" t="s">
         <v>221</v>
       </c>
-      <c r="G11" s="9" t="s">
-        <v>242</v>
-      </c>
-      <c r="H11" s="5" t="s">
+      <c r="G11" s="5" t="s">
         <v>232</v>
       </c>
     </row>
-    <row r="12" spans="1:8" ht="14.25" x14ac:dyDescent="0.45">
+    <row r="12" spans="1:7" ht="15" x14ac:dyDescent="0.25">
       <c r="A12" s="2">
         <v>11</v>
       </c>
@@ -1532,14 +1490,11 @@
       <c r="F12" s="9" t="s">
         <v>221</v>
       </c>
-      <c r="G12" s="9" t="s">
-        <v>242</v>
-      </c>
-      <c r="H12" s="5" t="s">
+      <c r="G12" s="5" t="s">
         <v>232</v>
       </c>
     </row>
-    <row r="13" spans="1:8" ht="14.25" x14ac:dyDescent="0.45">
+    <row r="13" spans="1:7" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A13" s="2">
         <v>12</v>
       </c>
@@ -1558,14 +1513,11 @@
       <c r="F13" s="9" t="s">
         <v>221</v>
       </c>
-      <c r="G13" s="9" t="s">
-        <v>242</v>
-      </c>
-      <c r="H13" s="5" t="s">
+      <c r="G13" s="5" t="s">
         <v>232</v>
       </c>
     </row>
-    <row r="14" spans="1:8" ht="14.25" x14ac:dyDescent="0.45">
+    <row r="14" spans="1:7" ht="15" x14ac:dyDescent="0.25">
       <c r="A14" s="2">
         <v>13</v>
       </c>
@@ -1584,14 +1536,11 @@
       <c r="F14" s="9" t="s">
         <v>221</v>
       </c>
-      <c r="G14" s="9" t="s">
-        <v>242</v>
-      </c>
-      <c r="H14" s="5" t="s">
+      <c r="G14" s="5" t="s">
         <v>232</v>
       </c>
     </row>
-    <row r="15" spans="1:8" ht="14.25" x14ac:dyDescent="0.45">
+    <row r="15" spans="1:7" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A15" s="2">
         <v>14</v>
       </c>
@@ -1610,14 +1559,11 @@
       <c r="F15" s="9" t="s">
         <v>221</v>
       </c>
-      <c r="G15" s="9" t="s">
-        <v>242</v>
-      </c>
-      <c r="H15" s="5" t="s">
+      <c r="G15" s="5" t="s">
         <v>232</v>
       </c>
     </row>
-    <row r="16" spans="1:8" ht="14.25" x14ac:dyDescent="0.45">
+    <row r="16" spans="1:7" ht="15" x14ac:dyDescent="0.25">
       <c r="A16" s="2">
         <v>15</v>
       </c>
@@ -1636,14 +1582,11 @@
       <c r="F16" s="9" t="s">
         <v>222</v>
       </c>
-      <c r="G16" s="9" t="s">
-        <v>222</v>
-      </c>
-      <c r="H16" s="5" t="s">
+      <c r="G16" s="5" t="s">
         <v>233</v>
       </c>
     </row>
-    <row r="17" spans="1:8" ht="14.25" x14ac:dyDescent="0.45">
+    <row r="17" spans="1:7" ht="15" x14ac:dyDescent="0.25">
       <c r="A17" s="2">
         <v>16</v>
       </c>
@@ -1662,14 +1605,11 @@
       <c r="F17" s="9" t="s">
         <v>222</v>
       </c>
-      <c r="G17" s="9" t="s">
-        <v>222</v>
-      </c>
-      <c r="H17" s="5" t="s">
+      <c r="G17" s="5" t="s">
         <v>233</v>
       </c>
     </row>
-    <row r="18" spans="1:8" ht="14.25" x14ac:dyDescent="0.45">
+    <row r="18" spans="1:7" ht="15" x14ac:dyDescent="0.25">
       <c r="A18" s="2">
         <v>17</v>
       </c>
@@ -1688,14 +1628,11 @@
       <c r="F18" s="9" t="s">
         <v>222</v>
       </c>
-      <c r="G18" s="9" t="s">
-        <v>222</v>
-      </c>
-      <c r="H18" s="5" t="s">
+      <c r="G18" s="5" t="s">
         <v>233</v>
       </c>
     </row>
-    <row r="19" spans="1:8" ht="14.25" x14ac:dyDescent="0.45">
+    <row r="19" spans="1:7" ht="15" x14ac:dyDescent="0.25">
       <c r="A19" s="2">
         <v>18</v>
       </c>
@@ -1714,14 +1651,11 @@
       <c r="F19" s="9" t="s">
         <v>222</v>
       </c>
-      <c r="G19" s="9" t="s">
-        <v>222</v>
-      </c>
-      <c r="H19" s="5" t="s">
+      <c r="G19" s="5" t="s">
         <v>233</v>
       </c>
     </row>
-    <row r="20" spans="1:8" ht="14.25" x14ac:dyDescent="0.45">
+    <row r="20" spans="1:7" ht="15" x14ac:dyDescent="0.25">
       <c r="A20" s="2">
         <v>19</v>
       </c>
@@ -1740,14 +1674,11 @@
       <c r="F20" s="9" t="s">
         <v>221</v>
       </c>
-      <c r="G20" s="9" t="s">
-        <v>242</v>
-      </c>
-      <c r="H20" s="5" t="s">
+      <c r="G20" s="5" t="s">
         <v>232</v>
       </c>
     </row>
-    <row r="21" spans="1:8" ht="14.25" x14ac:dyDescent="0.45">
+    <row r="21" spans="1:7" ht="15" x14ac:dyDescent="0.25">
       <c r="A21" s="2">
         <v>20</v>
       </c>
@@ -1766,14 +1697,11 @@
       <c r="F21" s="9" t="s">
         <v>222</v>
       </c>
-      <c r="G21" s="9" t="s">
-        <v>222</v>
-      </c>
-      <c r="H21" s="5" t="s">
+      <c r="G21" s="5" t="s">
         <v>233</v>
       </c>
     </row>
-    <row r="22" spans="1:8" ht="14.25" x14ac:dyDescent="0.45">
+    <row r="22" spans="1:7" ht="15" x14ac:dyDescent="0.25">
       <c r="A22" s="2">
         <v>21</v>
       </c>
@@ -1792,14 +1720,11 @@
       <c r="F22" s="9" t="s">
         <v>222</v>
       </c>
-      <c r="G22" s="9" t="s">
-        <v>222</v>
-      </c>
-      <c r="H22" s="5" t="s">
+      <c r="G22" s="5" t="s">
         <v>233</v>
       </c>
     </row>
-    <row r="23" spans="1:8" ht="14.25" x14ac:dyDescent="0.45">
+    <row r="23" spans="1:7" ht="15" x14ac:dyDescent="0.25">
       <c r="A23" s="2">
         <v>22</v>
       </c>
@@ -1818,14 +1743,11 @@
       <c r="F23" s="9" t="s">
         <v>222</v>
       </c>
-      <c r="G23" s="9" t="s">
-        <v>222</v>
-      </c>
-      <c r="H23" s="5" t="s">
+      <c r="G23" s="5" t="s">
         <v>233</v>
       </c>
     </row>
-    <row r="24" spans="1:8" ht="14.25" x14ac:dyDescent="0.45">
+    <row r="24" spans="1:7" ht="15" x14ac:dyDescent="0.25">
       <c r="A24" s="2">
         <v>23</v>
       </c>
@@ -1844,14 +1766,11 @@
       <c r="F24" s="9" t="s">
         <v>222</v>
       </c>
-      <c r="G24" s="9" t="s">
-        <v>222</v>
-      </c>
-      <c r="H24" s="5" t="s">
+      <c r="G24" s="5" t="s">
         <v>233</v>
       </c>
     </row>
-    <row r="25" spans="1:8" ht="14.25" x14ac:dyDescent="0.45">
+    <row r="25" spans="1:7" ht="15" x14ac:dyDescent="0.25">
       <c r="A25" s="2">
         <v>24</v>
       </c>
@@ -1870,14 +1789,11 @@
       <c r="F25" s="9" t="s">
         <v>222</v>
       </c>
-      <c r="G25" s="9" t="s">
-        <v>222</v>
-      </c>
-      <c r="H25" s="5" t="s">
+      <c r="G25" s="5" t="s">
         <v>233</v>
       </c>
     </row>
-    <row r="26" spans="1:8" ht="14.25" x14ac:dyDescent="0.45">
+    <row r="26" spans="1:7" ht="15" x14ac:dyDescent="0.25">
       <c r="A26" s="2">
         <v>25</v>
       </c>
@@ -1896,14 +1812,11 @@
       <c r="F26" s="9" t="s">
         <v>222</v>
       </c>
-      <c r="G26" s="9" t="s">
-        <v>222</v>
-      </c>
-      <c r="H26" s="5" t="s">
+      <c r="G26" s="5" t="s">
         <v>233</v>
       </c>
     </row>
-    <row r="27" spans="1:8" ht="26.25" x14ac:dyDescent="0.45">
+    <row r="27" spans="1:7" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A27" s="2">
         <v>26</v>
       </c>
@@ -1922,14 +1835,11 @@
       <c r="F27" s="9" t="s">
         <v>222</v>
       </c>
-      <c r="G27" s="9" t="s">
-        <v>222</v>
-      </c>
-      <c r="H27" s="5" t="s">
+      <c r="G27" s="5" t="s">
         <v>233</v>
       </c>
     </row>
-    <row r="28" spans="1:8" ht="14.25" x14ac:dyDescent="0.45">
+    <row r="28" spans="1:7" ht="15" x14ac:dyDescent="0.25">
       <c r="A28" s="2">
         <v>27</v>
       </c>
@@ -1948,14 +1858,11 @@
       <c r="F28" s="9" t="s">
         <v>222</v>
       </c>
-      <c r="G28" s="9" t="s">
-        <v>222</v>
-      </c>
-      <c r="H28" s="5" t="s">
+      <c r="G28" s="5" t="s">
         <v>233</v>
       </c>
     </row>
-    <row r="29" spans="1:8" ht="14.25" x14ac:dyDescent="0.45">
+    <row r="29" spans="1:7" ht="15" x14ac:dyDescent="0.25">
       <c r="A29" s="2">
         <v>28</v>
       </c>
@@ -1974,14 +1881,11 @@
       <c r="F29" s="9" t="s">
         <v>222</v>
       </c>
-      <c r="G29" s="9" t="s">
-        <v>222</v>
-      </c>
-      <c r="H29" s="5" t="s">
+      <c r="G29" s="5" t="s">
         <v>233</v>
       </c>
     </row>
-    <row r="30" spans="1:8" ht="14.25" x14ac:dyDescent="0.45">
+    <row r="30" spans="1:7" ht="15" x14ac:dyDescent="0.25">
       <c r="A30" s="2">
         <v>29</v>
       </c>
@@ -2000,14 +1904,11 @@
       <c r="F30" s="9" t="s">
         <v>221</v>
       </c>
-      <c r="G30" s="9" t="s">
-        <v>242</v>
-      </c>
-      <c r="H30" s="5" t="s">
+      <c r="G30" s="5" t="s">
         <v>232</v>
       </c>
     </row>
-    <row r="31" spans="1:8" ht="14.25" x14ac:dyDescent="0.45">
+    <row r="31" spans="1:7" ht="15" x14ac:dyDescent="0.25">
       <c r="A31" s="2">
         <v>30</v>
       </c>
@@ -2026,14 +1927,11 @@
       <c r="F31" s="9" t="s">
         <v>221</v>
       </c>
-      <c r="G31" s="9" t="s">
-        <v>242</v>
-      </c>
-      <c r="H31" s="5" t="s">
+      <c r="G31" s="5" t="s">
         <v>232</v>
       </c>
     </row>
-    <row r="32" spans="1:8" ht="14.25" x14ac:dyDescent="0.45">
+    <row r="32" spans="1:7" ht="15" x14ac:dyDescent="0.25">
       <c r="A32" s="2">
         <v>31</v>
       </c>
@@ -2052,14 +1950,11 @@
       <c r="F32" s="9" t="s">
         <v>221</v>
       </c>
-      <c r="G32" s="9" t="s">
-        <v>242</v>
-      </c>
-      <c r="H32" s="5" t="s">
+      <c r="G32" s="5" t="s">
         <v>232</v>
       </c>
     </row>
-    <row r="33" spans="1:8" ht="14.25" x14ac:dyDescent="0.45">
+    <row r="33" spans="1:7" ht="15" x14ac:dyDescent="0.25">
       <c r="A33" s="2">
         <v>32</v>
       </c>
@@ -2078,14 +1973,11 @@
       <c r="F33" s="9" t="s">
         <v>221</v>
       </c>
-      <c r="G33" s="9" t="s">
-        <v>242</v>
-      </c>
-      <c r="H33" s="5" t="s">
+      <c r="G33" s="5" t="s">
         <v>232</v>
       </c>
     </row>
-    <row r="34" spans="1:8" ht="14.25" x14ac:dyDescent="0.45">
+    <row r="34" spans="1:7" ht="15" x14ac:dyDescent="0.25">
       <c r="A34" s="2">
         <v>33</v>
       </c>
@@ -2104,14 +1996,11 @@
       <c r="F34" s="9" t="s">
         <v>221</v>
       </c>
-      <c r="G34" s="9" t="s">
-        <v>242</v>
-      </c>
-      <c r="H34" s="5" t="s">
+      <c r="G34" s="5" t="s">
         <v>232</v>
       </c>
     </row>
-    <row r="35" spans="1:8" ht="14.25" x14ac:dyDescent="0.45">
+    <row r="35" spans="1:7" ht="15" x14ac:dyDescent="0.25">
       <c r="A35" s="2">
         <v>34</v>
       </c>
@@ -2130,14 +2019,11 @@
       <c r="F35" s="9" t="s">
         <v>221</v>
       </c>
-      <c r="G35" s="9" t="s">
-        <v>242</v>
-      </c>
-      <c r="H35" s="5" t="s">
+      <c r="G35" s="5" t="s">
         <v>232</v>
       </c>
     </row>
-    <row r="36" spans="1:8" ht="14.25" x14ac:dyDescent="0.45">
+    <row r="36" spans="1:7" ht="15" x14ac:dyDescent="0.25">
       <c r="A36" s="2">
         <v>35</v>
       </c>
@@ -2156,14 +2042,11 @@
       <c r="F36" s="9" t="s">
         <v>221</v>
       </c>
-      <c r="G36" s="9" t="s">
-        <v>242</v>
-      </c>
-      <c r="H36" s="5" t="s">
+      <c r="G36" s="5" t="s">
         <v>232</v>
       </c>
     </row>
-    <row r="37" spans="1:8" ht="14.25" x14ac:dyDescent="0.45">
+    <row r="37" spans="1:7" ht="15" x14ac:dyDescent="0.25">
       <c r="A37" s="2">
         <v>36</v>
       </c>
@@ -2182,14 +2065,11 @@
       <c r="F37" s="9" t="s">
         <v>221</v>
       </c>
-      <c r="G37" s="9" t="s">
-        <v>242</v>
-      </c>
-      <c r="H37" s="5" t="s">
+      <c r="G37" s="5" t="s">
         <v>232</v>
       </c>
     </row>
-    <row r="38" spans="1:8" ht="14.25" x14ac:dyDescent="0.45">
+    <row r="38" spans="1:7" ht="15" x14ac:dyDescent="0.25">
       <c r="A38" s="2">
         <v>37</v>
       </c>
@@ -2208,14 +2088,11 @@
       <c r="F38" s="9" t="s">
         <v>223</v>
       </c>
-      <c r="G38" s="9" t="s">
-        <v>223</v>
-      </c>
-      <c r="H38" s="5" t="s">
+      <c r="G38" s="5" t="s">
         <v>234</v>
       </c>
     </row>
-    <row r="39" spans="1:8" ht="14.25" x14ac:dyDescent="0.45">
+    <row r="39" spans="1:7" ht="15" x14ac:dyDescent="0.25">
       <c r="A39" s="2">
         <v>38</v>
       </c>
@@ -2234,14 +2111,11 @@
       <c r="F39" s="9" t="s">
         <v>223</v>
       </c>
-      <c r="G39" s="9" t="s">
-        <v>223</v>
-      </c>
-      <c r="H39" s="5" t="s">
+      <c r="G39" s="5" t="s">
         <v>234</v>
       </c>
     </row>
-    <row r="40" spans="1:8" ht="14.25" x14ac:dyDescent="0.45">
+    <row r="40" spans="1:7" ht="15" x14ac:dyDescent="0.25">
       <c r="A40" s="2">
         <v>39</v>
       </c>
@@ -2260,14 +2134,11 @@
       <c r="F40" s="9" t="s">
         <v>223</v>
       </c>
-      <c r="G40" s="9" t="s">
-        <v>223</v>
-      </c>
-      <c r="H40" s="5" t="s">
+      <c r="G40" s="5" t="s">
         <v>234</v>
       </c>
     </row>
-    <row r="41" spans="1:8" ht="14.25" x14ac:dyDescent="0.45">
+    <row r="41" spans="1:7" ht="15" x14ac:dyDescent="0.25">
       <c r="A41" s="2">
         <v>40</v>
       </c>
@@ -2286,14 +2157,11 @@
       <c r="F41" s="9" t="s">
         <v>223</v>
       </c>
-      <c r="G41" s="9" t="s">
-        <v>223</v>
-      </c>
-      <c r="H41" s="5" t="s">
+      <c r="G41" s="5" t="s">
         <v>234</v>
       </c>
     </row>
-    <row r="42" spans="1:8" ht="14.25" x14ac:dyDescent="0.45">
+    <row r="42" spans="1:7" ht="15" x14ac:dyDescent="0.25">
       <c r="A42" s="2">
         <v>41</v>
       </c>
@@ -2312,14 +2180,11 @@
       <c r="F42" s="9" t="s">
         <v>224</v>
       </c>
-      <c r="G42" s="9" t="s">
-        <v>224</v>
-      </c>
-      <c r="H42" s="5" t="s">
+      <c r="G42" s="5" t="s">
         <v>235</v>
       </c>
     </row>
-    <row r="43" spans="1:8" ht="14.25" x14ac:dyDescent="0.45">
+    <row r="43" spans="1:7" ht="15" x14ac:dyDescent="0.25">
       <c r="A43" s="2">
         <v>42</v>
       </c>
@@ -2338,14 +2203,11 @@
       <c r="F43" s="9" t="s">
         <v>225</v>
       </c>
-      <c r="G43" s="9" t="s">
-        <v>225</v>
-      </c>
-      <c r="H43" s="5" t="s">
+      <c r="G43" s="5" t="s">
         <v>236</v>
       </c>
     </row>
-    <row r="44" spans="1:8" ht="14.25" x14ac:dyDescent="0.45">
+    <row r="44" spans="1:7" ht="15" x14ac:dyDescent="0.25">
       <c r="A44" s="2">
         <v>43</v>
       </c>
@@ -2364,14 +2226,11 @@
       <c r="F44" s="9" t="s">
         <v>225</v>
       </c>
-      <c r="G44" s="9" t="s">
-        <v>225</v>
-      </c>
-      <c r="H44" s="5" t="s">
+      <c r="G44" s="5" t="s">
         <v>236</v>
       </c>
     </row>
-    <row r="45" spans="1:8" ht="14.25" x14ac:dyDescent="0.45">
+    <row r="45" spans="1:7" ht="15" x14ac:dyDescent="0.25">
       <c r="A45" s="2">
         <v>44</v>
       </c>
@@ -2390,14 +2249,11 @@
       <c r="F45" s="9" t="s">
         <v>225</v>
       </c>
-      <c r="G45" s="9" t="s">
-        <v>225</v>
-      </c>
-      <c r="H45" s="5" t="s">
+      <c r="G45" s="5" t="s">
         <v>236</v>
       </c>
     </row>
-    <row r="46" spans="1:8" ht="14.25" x14ac:dyDescent="0.45">
+    <row r="46" spans="1:7" ht="15" x14ac:dyDescent="0.25">
       <c r="A46" s="2">
         <v>45</v>
       </c>
@@ -2416,14 +2272,11 @@
       <c r="F46" s="9" t="s">
         <v>225</v>
       </c>
-      <c r="G46" s="9" t="s">
-        <v>225</v>
-      </c>
-      <c r="H46" s="5" t="s">
+      <c r="G46" s="5" t="s">
         <v>236</v>
       </c>
     </row>
-    <row r="47" spans="1:8" ht="14.25" x14ac:dyDescent="0.45">
+    <row r="47" spans="1:7" ht="15" x14ac:dyDescent="0.25">
       <c r="A47" s="2">
         <v>46</v>
       </c>
@@ -2442,14 +2295,11 @@
       <c r="F47" s="9" t="s">
         <v>226</v>
       </c>
-      <c r="G47" s="9" t="s">
-        <v>226</v>
-      </c>
-      <c r="H47" s="5" t="s">
+      <c r="G47" s="5" t="s">
         <v>237</v>
       </c>
     </row>
-    <row r="48" spans="1:8" ht="14.25" x14ac:dyDescent="0.45">
+    <row r="48" spans="1:7" ht="15" x14ac:dyDescent="0.25">
       <c r="A48" s="2">
         <v>47</v>
       </c>
@@ -2468,14 +2318,11 @@
       <c r="F48" s="9" t="s">
         <v>226</v>
       </c>
-      <c r="G48" s="9" t="s">
-        <v>226</v>
-      </c>
-      <c r="H48" s="5" t="s">
+      <c r="G48" s="5" t="s">
         <v>237</v>
       </c>
     </row>
-    <row r="49" spans="1:8" ht="14.25" x14ac:dyDescent="0.45">
+    <row r="49" spans="1:7" ht="15" x14ac:dyDescent="0.25">
       <c r="A49" s="2">
         <v>48</v>
       </c>
@@ -2494,14 +2341,11 @@
       <c r="F49" s="9" t="s">
         <v>226</v>
       </c>
-      <c r="G49" s="9" t="s">
-        <v>226</v>
-      </c>
-      <c r="H49" s="5" t="s">
+      <c r="G49" s="5" t="s">
         <v>237</v>
       </c>
     </row>
-    <row r="50" spans="1:8" ht="14.25" x14ac:dyDescent="0.45">
+    <row r="50" spans="1:7" ht="15" x14ac:dyDescent="0.25">
       <c r="A50" s="2">
         <v>49</v>
       </c>
@@ -2520,14 +2364,11 @@
       <c r="F50" s="9" t="s">
         <v>226</v>
       </c>
-      <c r="G50" s="9" t="s">
-        <v>226</v>
-      </c>
-      <c r="H50" s="5" t="s">
+      <c r="G50" s="5" t="s">
         <v>237</v>
       </c>
     </row>
-    <row r="51" spans="1:8" ht="14.25" x14ac:dyDescent="0.45">
+    <row r="51" spans="1:7" ht="15" x14ac:dyDescent="0.25">
       <c r="A51" s="2">
         <v>50</v>
       </c>
@@ -2546,14 +2387,11 @@
       <c r="F51" s="9" t="s">
         <v>227</v>
       </c>
-      <c r="G51" s="9" t="s">
-        <v>227</v>
-      </c>
-      <c r="H51" s="5" t="s">
+      <c r="G51" s="5" t="s">
         <v>238</v>
       </c>
     </row>
-    <row r="52" spans="1:8" ht="14.25" x14ac:dyDescent="0.45">
+    <row r="52" spans="1:7" ht="15" x14ac:dyDescent="0.25">
       <c r="A52" s="2">
         <v>51</v>
       </c>
@@ -2572,14 +2410,11 @@
       <c r="F52" s="9" t="s">
         <v>227</v>
       </c>
-      <c r="G52" s="9" t="s">
-        <v>227</v>
-      </c>
-      <c r="H52" s="5" t="s">
+      <c r="G52" s="5" t="s">
         <v>238</v>
       </c>
     </row>
-    <row r="53" spans="1:8" ht="14.25" x14ac:dyDescent="0.45">
+    <row r="53" spans="1:7" ht="15" x14ac:dyDescent="0.25">
       <c r="A53" s="2">
         <v>52</v>
       </c>
@@ -2598,14 +2433,11 @@
       <c r="F53" s="9" t="s">
         <v>227</v>
       </c>
-      <c r="G53" s="9" t="s">
-        <v>227</v>
-      </c>
-      <c r="H53" s="5" t="s">
+      <c r="G53" s="5" t="s">
         <v>238</v>
       </c>
     </row>
-    <row r="54" spans="1:8" ht="14.25" x14ac:dyDescent="0.45">
+    <row r="54" spans="1:7" ht="15" x14ac:dyDescent="0.25">
       <c r="A54" s="2">
         <v>53</v>
       </c>
@@ -2624,14 +2456,11 @@
       <c r="F54" s="9" t="s">
         <v>227</v>
       </c>
-      <c r="G54" s="9" t="s">
-        <v>227</v>
-      </c>
-      <c r="H54" s="5" t="s">
+      <c r="G54" s="5" t="s">
         <v>238</v>
       </c>
     </row>
-    <row r="55" spans="1:8" ht="14.25" x14ac:dyDescent="0.45">
+    <row r="55" spans="1:7" ht="15" x14ac:dyDescent="0.25">
       <c r="A55" s="2">
         <v>54</v>
       </c>
@@ -2650,14 +2479,11 @@
       <c r="F55" s="9" t="s">
         <v>228</v>
       </c>
-      <c r="G55" s="9" t="s">
-        <v>228</v>
-      </c>
-      <c r="H55" s="5" t="s">
+      <c r="G55" s="5" t="s">
         <v>239</v>
       </c>
     </row>
-    <row r="56" spans="1:8" ht="14.25" x14ac:dyDescent="0.45">
+    <row r="56" spans="1:7" ht="15" x14ac:dyDescent="0.25">
       <c r="A56" s="2">
         <v>55</v>
       </c>
@@ -2676,14 +2502,11 @@
       <c r="F56" s="9" t="s">
         <v>228</v>
       </c>
-      <c r="G56" s="9" t="s">
-        <v>228</v>
-      </c>
-      <c r="H56" s="5" t="s">
+      <c r="G56" s="5" t="s">
         <v>239</v>
       </c>
     </row>
-    <row r="57" spans="1:8" ht="14.25" x14ac:dyDescent="0.45">
+    <row r="57" spans="1:7" ht="15" x14ac:dyDescent="0.25">
       <c r="A57" s="2">
         <v>56</v>
       </c>
@@ -2702,14 +2525,11 @@
       <c r="F57" s="9" t="s">
         <v>228</v>
       </c>
-      <c r="G57" s="9" t="s">
-        <v>228</v>
-      </c>
-      <c r="H57" s="5" t="s">
+      <c r="G57" s="5" t="s">
         <v>239</v>
       </c>
     </row>
-    <row r="58" spans="1:8" ht="14.25" x14ac:dyDescent="0.45">
+    <row r="58" spans="1:7" ht="15" x14ac:dyDescent="0.25">
       <c r="A58" s="2">
         <v>57</v>
       </c>
@@ -2728,14 +2548,11 @@
       <c r="F58" s="9" t="s">
         <v>227</v>
       </c>
-      <c r="G58" s="9" t="s">
-        <v>227</v>
-      </c>
-      <c r="H58" s="5" t="s">
+      <c r="G58" s="5" t="s">
         <v>238</v>
       </c>
     </row>
-    <row r="59" spans="1:8" ht="14.25" x14ac:dyDescent="0.45">
+    <row r="59" spans="1:7" ht="15" x14ac:dyDescent="0.25">
       <c r="A59" s="2">
         <v>58</v>
       </c>
@@ -2754,14 +2571,11 @@
       <c r="F59" s="9" t="s">
         <v>228</v>
       </c>
-      <c r="G59" s="9" t="s">
-        <v>228</v>
-      </c>
-      <c r="H59" s="5" t="s">
+      <c r="G59" s="5" t="s">
         <v>239</v>
       </c>
     </row>
-    <row r="60" spans="1:8" ht="14.25" x14ac:dyDescent="0.45">
+    <row r="60" spans="1:7" ht="15" x14ac:dyDescent="0.25">
       <c r="A60" s="2">
         <v>59</v>
       </c>
@@ -2780,14 +2594,11 @@
       <c r="F60" s="9" t="s">
         <v>228</v>
       </c>
-      <c r="G60" s="9" t="s">
-        <v>228</v>
-      </c>
-      <c r="H60" s="5" t="s">
+      <c r="G60" s="5" t="s">
         <v>239</v>
       </c>
     </row>
-    <row r="61" spans="1:8" ht="14.25" x14ac:dyDescent="0.45">
+    <row r="61" spans="1:7" ht="15" x14ac:dyDescent="0.25">
       <c r="A61" s="2">
         <v>60</v>
       </c>
@@ -2806,14 +2617,11 @@
       <c r="F61" s="9" t="s">
         <v>228</v>
       </c>
-      <c r="G61" s="9" t="s">
-        <v>228</v>
-      </c>
-      <c r="H61" s="5" t="s">
+      <c r="G61" s="5" t="s">
         <v>239</v>
       </c>
     </row>
-    <row r="62" spans="1:8" ht="14.25" x14ac:dyDescent="0.45">
+    <row r="62" spans="1:7" ht="15" x14ac:dyDescent="0.25">
       <c r="A62" s="2">
         <v>61</v>
       </c>
@@ -2832,14 +2640,11 @@
       <c r="F62" s="9" t="s">
         <v>222</v>
       </c>
-      <c r="G62" s="9" t="s">
-        <v>222</v>
-      </c>
-      <c r="H62" s="5" t="s">
+      <c r="G62" s="5" t="s">
         <v>233</v>
       </c>
     </row>
-    <row r="63" spans="1:8" ht="14.25" x14ac:dyDescent="0.45">
+    <row r="63" spans="1:7" ht="15" x14ac:dyDescent="0.25">
       <c r="A63" s="2">
         <v>62</v>
       </c>
@@ -2858,14 +2663,11 @@
       <c r="F63" s="9" t="s">
         <v>222</v>
       </c>
-      <c r="G63" s="9" t="s">
-        <v>222</v>
-      </c>
-      <c r="H63" s="5" t="s">
+      <c r="G63" s="5" t="s">
         <v>233</v>
       </c>
     </row>
-    <row r="64" spans="1:8" ht="14.25" x14ac:dyDescent="0.45">
+    <row r="64" spans="1:7" ht="15" x14ac:dyDescent="0.25">
       <c r="A64" s="2">
         <v>63</v>
       </c>
@@ -2884,14 +2686,11 @@
       <c r="F64" s="9" t="s">
         <v>222</v>
       </c>
-      <c r="G64" s="9" t="s">
-        <v>222</v>
-      </c>
-      <c r="H64" s="5" t="s">
+      <c r="G64" s="5" t="s">
         <v>233</v>
       </c>
     </row>
-    <row r="65" spans="1:8" ht="14.25" x14ac:dyDescent="0.45">
+    <row r="65" spans="1:7" ht="15" x14ac:dyDescent="0.25">
       <c r="A65" s="2">
         <v>64</v>
       </c>
@@ -2910,14 +2709,11 @@
       <c r="F65" s="9" t="s">
         <v>229</v>
       </c>
-      <c r="G65" s="9" t="s">
-        <v>243</v>
-      </c>
-      <c r="H65" s="5" t="s">
+      <c r="G65" s="5" t="s">
         <v>240</v>
       </c>
     </row>
-    <row r="66" spans="1:8" ht="14.25" x14ac:dyDescent="0.45">
+    <row r="66" spans="1:7" ht="15" x14ac:dyDescent="0.25">
       <c r="A66" s="2">
         <v>65</v>
       </c>
@@ -2936,14 +2732,11 @@
       <c r="F66" s="9" t="s">
         <v>229</v>
       </c>
-      <c r="G66" s="9" t="s">
-        <v>243</v>
-      </c>
-      <c r="H66" s="5" t="s">
+      <c r="G66" s="5" t="s">
         <v>240</v>
       </c>
     </row>
-    <row r="67" spans="1:8" ht="26.25" x14ac:dyDescent="0.45">
+    <row r="67" spans="1:7" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A67" s="2">
         <v>66</v>
       </c>
@@ -2962,14 +2755,11 @@
       <c r="F67" s="9" t="s">
         <v>222</v>
       </c>
-      <c r="G67" s="9" t="s">
-        <v>222</v>
-      </c>
-      <c r="H67" s="5" t="s">
+      <c r="G67" s="5" t="s">
         <v>233</v>
       </c>
     </row>
-    <row r="68" spans="1:8" ht="14.25" x14ac:dyDescent="0.45">
+    <row r="68" spans="1:7" ht="15" x14ac:dyDescent="0.25">
       <c r="A68" s="2">
         <v>67</v>
       </c>
@@ -2988,14 +2778,11 @@
       <c r="F68" s="9" t="s">
         <v>222</v>
       </c>
-      <c r="G68" s="9" t="s">
-        <v>222</v>
-      </c>
-      <c r="H68" s="5" t="s">
+      <c r="G68" s="5" t="s">
         <v>233</v>
       </c>
     </row>
-    <row r="69" spans="1:8" ht="14.25" x14ac:dyDescent="0.45">
+    <row r="69" spans="1:7" ht="15" x14ac:dyDescent="0.25">
       <c r="A69" s="2">
         <v>68</v>
       </c>
@@ -3014,14 +2801,11 @@
       <c r="F69" s="9" t="s">
         <v>222</v>
       </c>
-      <c r="G69" s="9" t="s">
-        <v>222</v>
-      </c>
-      <c r="H69" s="5" t="s">
+      <c r="G69" s="5" t="s">
         <v>233</v>
       </c>
     </row>
-    <row r="70" spans="1:8" ht="14.25" x14ac:dyDescent="0.45">
+    <row r="70" spans="1:7" ht="15" x14ac:dyDescent="0.25">
       <c r="A70" s="2">
         <v>69</v>
       </c>
@@ -3040,14 +2824,11 @@
       <c r="F70" s="9" t="s">
         <v>222</v>
       </c>
-      <c r="G70" s="9" t="s">
-        <v>222</v>
-      </c>
-      <c r="H70" s="5" t="s">
+      <c r="G70" s="5" t="s">
         <v>233</v>
       </c>
     </row>
-    <row r="71" spans="1:8" ht="14.25" x14ac:dyDescent="0.45">
+    <row r="71" spans="1:7" ht="15" x14ac:dyDescent="0.25">
       <c r="A71" s="2">
         <v>70</v>
       </c>
@@ -3066,14 +2847,11 @@
       <c r="F71" s="9" t="s">
         <v>222</v>
       </c>
-      <c r="G71" s="9" t="s">
-        <v>222</v>
-      </c>
-      <c r="H71" s="5" t="s">
+      <c r="G71" s="5" t="s">
         <v>233</v>
       </c>
     </row>
-    <row r="72" spans="1:8" ht="14.25" x14ac:dyDescent="0.45">
+    <row r="72" spans="1:7" ht="15" x14ac:dyDescent="0.25">
       <c r="A72" s="2">
         <v>71</v>
       </c>
@@ -3092,14 +2870,11 @@
       <c r="F72" s="9" t="s">
         <v>222</v>
       </c>
-      <c r="G72" s="9" t="s">
-        <v>222</v>
-      </c>
-      <c r="H72" s="5" t="s">
+      <c r="G72" s="5" t="s">
         <v>233</v>
       </c>
     </row>
-    <row r="73" spans="1:8" ht="14.25" x14ac:dyDescent="0.45">
+    <row r="73" spans="1:7" ht="15" x14ac:dyDescent="0.25">
       <c r="A73" s="2">
         <v>72</v>
       </c>
@@ -3118,10 +2893,7 @@
       <c r="F73" s="9" t="s">
         <v>230</v>
       </c>
-      <c r="G73" s="9" t="s">
-        <v>230</v>
-      </c>
-      <c r="H73" s="5" t="s">
+      <c r="G73" s="5" t="s">
         <v>230</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Ensemble update - Introduce EI Interventions - Add patch identification - Outsource R code from the Dinamica model - Use bash variables - Remove superfluous files
</commit_message>
<xml_diff>
--- a/tools/lulc_class_aggregation.xlsx
+++ b/tools/lulc_class_aggregation.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="26924"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="27231"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\bblack\switchdrive\C.3_Modelling\LULCC_CH_HPC\Tools\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\LULCC_CH_Ensemble\Tools\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FB7150C2-BB2F-41DF-8002-A52E3EBAB9A4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7AD4D755-52C1-4D61-A62D-2222CD546612}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{461A3D3D-11BC-4F5B-AC99-BB9F607AA1FC}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{461A3D3D-11BC-4F5B-AC99-BB9F607AA1FC}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>

</xml_diff>